<commit_message>
Recalibrate candidate storefront rents for Taiwan and KL
</commit_message>
<xml_diff>
--- a/salon_data.xlsx
+++ b/salon_data.xlsx
@@ -2064,7 +2064,7 @@
         <v>0.1</v>
       </c>
       <c r="J11" s="20" t="n">
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="K11" s="20" t="n">
         <v>33000</v>
@@ -2794,7 +2794,7 @@
         <v>0.1</v>
       </c>
       <c r="J21" s="20" t="n">
-        <v>2200</v>
+        <v>3400</v>
       </c>
       <c r="K21" s="20" t="n">
         <v>55800</v>
@@ -2867,7 +2867,7 @@
         <v>0.1</v>
       </c>
       <c r="J22" s="20" t="n">
-        <v>1800</v>
+        <v>3000</v>
       </c>
       <c r="K22" s="20" t="n">
         <v>46500</v>
@@ -2940,7 +2940,7 @@
         <v>0.1</v>
       </c>
       <c r="J23" s="20" t="n">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="K23" s="20" t="n">
         <v>37200</v>
@@ -3013,7 +3013,7 @@
         <v>0.1</v>
       </c>
       <c r="J24" s="20" t="n">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="K24" s="20" t="n">
         <v>34100</v>

</xml_diff>

<commit_message>
Implement foreign ownership legal context, tax compliance, and map cross-filtering
</commit_message>
<xml_diff>
--- a/salon_data.xlsx
+++ b/salon_data.xlsx
@@ -123,7 +123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -145,11 +145,55 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -236,6 +280,8 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1390,7 +1436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1436,36 +1482,50 @@
           <t>IDENTITY</t>
         </is>
       </c>
+      <c r="B3" s="30" t="n"/>
+      <c r="C3" s="30" t="n"/>
+      <c r="D3" s="31" t="n"/>
       <c r="E3" s="14" t="inlineStr">
         <is>
           <t>SPACE &amp; TIME</t>
         </is>
       </c>
+      <c r="F3" s="30" t="n"/>
+      <c r="G3" s="31" t="n"/>
       <c r="H3" s="14" t="inlineStr">
         <is>
           <t>PRICING</t>
         </is>
       </c>
+      <c r="I3" s="31" t="n"/>
       <c r="J3" s="14" t="inlineStr">
         <is>
           <t>COSTS &amp; CAPEX</t>
         </is>
       </c>
+      <c r="K3" s="30" t="n"/>
+      <c r="L3" s="30" t="n"/>
+      <c r="M3" s="30" t="n"/>
+      <c r="N3" s="31" t="n"/>
       <c r="O3" s="14" t="inlineStr">
         <is>
           <t>UTILISATION</t>
         </is>
       </c>
+      <c r="P3" s="31" t="n"/>
       <c r="Q3" s="14" t="inlineStr">
         <is>
           <t>GEOGRAPHY</t>
         </is>
       </c>
+      <c r="R3" s="30" t="n"/>
+      <c r="S3" s="31" t="n"/>
       <c r="T3" s="14" t="inlineStr">
         <is>
           <t>BUSINESS FEES &amp; ADMIN</t>
         </is>
       </c>
+      <c r="U3" s="31" t="n"/>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1656,7 +1716,7 @@
         <v>65</v>
       </c>
       <c r="T5" s="20" t="n">
-        <v>2500</v>
+        <v>6500</v>
       </c>
       <c r="U5" s="20" t="n">
         <v>200</v>
@@ -1729,7 +1789,7 @@
         <v>55</v>
       </c>
       <c r="T6" s="20" t="n">
-        <v>2500</v>
+        <v>6500</v>
       </c>
       <c r="U6" s="20" t="n">
         <v>200</v>
@@ -1802,7 +1862,7 @@
         <v>70</v>
       </c>
       <c r="T7" s="20" t="n">
-        <v>1500</v>
+        <v>6500</v>
       </c>
       <c r="U7" s="20" t="n">
         <v>200</v>
@@ -1875,7 +1935,7 @@
         <v>72</v>
       </c>
       <c r="T8" s="20" t="n">
-        <v>1500</v>
+        <v>6500</v>
       </c>
       <c r="U8" s="20" t="n">
         <v>200</v>
@@ -1948,7 +2008,7 @@
         <v>75</v>
       </c>
       <c r="T9" s="20" t="n">
-        <v>1500</v>
+        <v>6500</v>
       </c>
       <c r="U9" s="20" t="n">
         <v>200</v>
@@ -2021,7 +2081,7 @@
         <v>73</v>
       </c>
       <c r="T10" s="20" t="n">
-        <v>1500</v>
+        <v>6500</v>
       </c>
       <c r="U10" s="20" t="n">
         <v>200</v>
@@ -2094,7 +2154,7 @@
         <v>40</v>
       </c>
       <c r="T11" s="20" t="n">
-        <v>1500</v>
+        <v>7500</v>
       </c>
       <c r="U11" s="20" t="n">
         <v>200</v>
@@ -2167,7 +2227,7 @@
         <v>55</v>
       </c>
       <c r="T12" s="20" t="n">
-        <v>1500</v>
+        <v>7500</v>
       </c>
       <c r="U12" s="20" t="n">
         <v>200</v>
@@ -2240,7 +2300,7 @@
         <v>50</v>
       </c>
       <c r="T13" s="20" t="n">
-        <v>1000</v>
+        <v>7500</v>
       </c>
       <c r="U13" s="20" t="n">
         <v>200</v>
@@ -2313,7 +2373,7 @@
         <v>68</v>
       </c>
       <c r="T14" s="20" t="n">
-        <v>1000</v>
+        <v>7500</v>
       </c>
       <c r="U14" s="20" t="n">
         <v>200</v>
@@ -2386,7 +2446,7 @@
         <v>65</v>
       </c>
       <c r="T15" s="20" t="n">
-        <v>1000</v>
+        <v>7500</v>
       </c>
       <c r="U15" s="20" t="n">
         <v>200</v>
@@ -2459,7 +2519,7 @@
         <v>25</v>
       </c>
       <c r="T16" s="20" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="U16" s="20" t="n">
         <v>300</v>
@@ -2532,7 +2592,7 @@
         <v>22</v>
       </c>
       <c r="T17" s="20" t="n">
-        <v>1200</v>
+        <v>3500</v>
       </c>
       <c r="U17" s="20" t="n">
         <v>300</v>
@@ -2605,7 +2665,7 @@
         <v>45</v>
       </c>
       <c r="T18" s="20" t="n">
-        <v>2000</v>
+        <v>6500</v>
       </c>
       <c r="U18" s="20" t="n">
         <v>200</v>
@@ -2678,7 +2738,7 @@
         <v>38</v>
       </c>
       <c r="T19" s="20" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="U19" s="20" t="n">
         <v>300</v>
@@ -2751,7 +2811,7 @@
         <v>30</v>
       </c>
       <c r="T20" s="20" t="n">
-        <v>6000</v>
+        <v>8500</v>
       </c>
       <c r="U20" s="20" t="n">
         <v>300</v>
@@ -2824,7 +2884,7 @@
         <v>35</v>
       </c>
       <c r="T21" s="20" t="n">
-        <v>1800</v>
+        <v>5500</v>
       </c>
       <c r="U21" s="20" t="n">
         <v>200</v>
@@ -2897,7 +2957,7 @@
         <v>42</v>
       </c>
       <c r="T22" s="20" t="n">
-        <v>1800</v>
+        <v>5500</v>
       </c>
       <c r="U22" s="20" t="n">
         <v>200</v>
@@ -2970,7 +3030,7 @@
         <v>48</v>
       </c>
       <c r="T23" s="20" t="n">
-        <v>1800</v>
+        <v>5500</v>
       </c>
       <c r="U23" s="20" t="n">
         <v>200</v>
@@ -3043,7 +3103,7 @@
         <v>55</v>
       </c>
       <c r="T24" s="20" t="n">
-        <v>1800</v>
+        <v>5500</v>
       </c>
       <c r="U24" s="20" t="n">
         <v>200</v>
@@ -3116,7 +3176,7 @@
         <v>38</v>
       </c>
       <c r="T25" s="20" t="n">
-        <v>2500</v>
+        <v>7500</v>
       </c>
       <c r="U25" s="20" t="n">
         <v>300</v>
@@ -3189,7 +3249,7 @@
         <v>52</v>
       </c>
       <c r="T26" s="20" t="n">
-        <v>2500</v>
+        <v>7500</v>
       </c>
       <c r="U26" s="20" t="n">
         <v>300</v>
@@ -3262,7 +3322,7 @@
         <v>45</v>
       </c>
       <c r="T27" s="20" t="n">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="U27" s="20" t="n">
         <v>300</v>
@@ -3335,7 +3395,7 @@
         <v>30</v>
       </c>
       <c r="T28" s="20" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="U28" s="20" t="n">
         <v>300</v>
@@ -3408,7 +3468,7 @@
         <v>32</v>
       </c>
       <c r="T29" s="20" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="U29" s="20" t="n">
         <v>300</v>
@@ -3481,7 +3541,7 @@
         <v>36</v>
       </c>
       <c r="T30" s="20" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="U30" s="20" t="n">
         <v>300</v>
@@ -3554,12 +3614,30 @@
         <v>38</v>
       </c>
       <c r="T31" s="20" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="U31" s="20" t="n">
         <v>300</v>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="O3:P3"/>
@@ -3645,21 +3723,32 @@
           <t>IDENTITY</t>
         </is>
       </c>
+      <c r="B3" s="31" t="n"/>
       <c r="C3" s="14" t="inlineStr">
         <is>
           <t>SPACE &amp; SEATS</t>
         </is>
       </c>
+      <c r="D3" s="30" t="n"/>
+      <c r="E3" s="31" t="n"/>
       <c r="F3" s="14" t="inlineStr">
         <is>
           <t>STAFFING MODEL</t>
         </is>
       </c>
+      <c r="G3" s="30" t="n"/>
+      <c r="H3" s="30" t="n"/>
+      <c r="I3" s="30" t="n"/>
+      <c r="J3" s="31" t="n"/>
       <c r="K3" s="14" t="inlineStr">
         <is>
           <t>COUNTRY RATES</t>
         </is>
       </c>
+      <c r="L3" s="30" t="n"/>
+      <c r="M3" s="30" t="n"/>
+      <c r="N3" s="30" t="n"/>
+      <c r="O3" s="31" t="n"/>
       <c r="P3" s="14" t="inlineStr">
         <is>
           <t>STAFF COST</t>
@@ -3670,26 +3759,41 @@
           <t>MONTHLY OPEX</t>
         </is>
       </c>
+      <c r="R3" s="30" t="n"/>
+      <c r="S3" s="30" t="n"/>
+      <c r="T3" s="30" t="n"/>
+      <c r="U3" s="30" t="n"/>
+      <c r="V3" s="31" t="n"/>
       <c r="W3" s="14" t="inlineStr">
         <is>
           <t>CAPACITY</t>
         </is>
       </c>
+      <c r="X3" s="30" t="n"/>
+      <c r="Y3" s="31" t="n"/>
       <c r="Z3" s="14" t="inlineStr">
         <is>
           <t>UNIT ECONOMICS</t>
         </is>
       </c>
+      <c r="AA3" s="30" t="n"/>
+      <c r="AB3" s="31" t="n"/>
       <c r="AC3" s="14" t="inlineStr">
         <is>
           <t>PROFIT &amp; CASH FLOW</t>
         </is>
       </c>
+      <c r="AD3" s="30" t="n"/>
+      <c r="AE3" s="30" t="n"/>
+      <c r="AF3" s="31" t="n"/>
       <c r="AG3" s="14" t="inlineStr">
         <is>
           <t>CAPEX &amp; PAYBACK</t>
         </is>
       </c>
+      <c r="AH3" s="30" t="n"/>
+      <c r="AI3" s="30" t="n"/>
+      <c r="AJ3" s="31" t="n"/>
       <c r="AK3" s="14" t="inlineStr">
         <is>
           <t>RATIO</t>

</xml_diff>

<commit_message>
Audit competitors: Replace closed Kimrobinson in HK with SHHH (Hollywood Road), update capacity & note for Central Candidate B, update salon_data.xlsx cell S17, and convert Google Maps links to named search queries across all 27 subpages
</commit_message>
<xml_diff>
--- a/salon_data.xlsx
+++ b/salon_data.xlsx
@@ -1436,7 +1436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U49"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2589,7 +2589,7 @@
         <v>114.165</v>
       </c>
       <c r="S17" s="19" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="T17" s="20" t="n">
         <v>3500</v>
@@ -3620,24 +3620,6 @@
         <v>300</v>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="O3:P3"/>

</xml_diff>

<commit_message>
Implement interactive equipment sourcing analysis and inventory stock lists on subpages, backed by new Excel sheets
</commit_message>
<xml_diff>
--- a/salon_data.xlsx
+++ b/salon_data.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX_Details" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPEX_Details" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment_Sourcing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_Details" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -990,7 +992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1415,7 +1417,6 @@
         <v>3808</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
@@ -1423,10 +1424,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A16:H16"/>
@@ -1443,7 +1440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U50"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3627,25 +3624,6 @@
         <v>300</v>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="O3:P3"/>
@@ -24496,4 +24474,1500 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Equipment Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Import Model</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Import Base Cost (USD)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Logistics &amp; Duty (USD)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Total Import Cost (USD)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Local Supplier Model</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Local Supplier Cost (USD)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Cheaper Option</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Sourcing References &amp; Quotes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>180</v>
+      </c>
+      <c r="E2" t="n">
+        <v>129</v>
+      </c>
+      <c r="F2" t="n">
+        <v>309</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Hieu Salon Equipment Saigon</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>450</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Foshan factory quote &amp; local customs broker clearance estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>350</v>
+      </c>
+      <c r="E3" t="n">
+        <v>255</v>
+      </c>
+      <c r="F3" t="n">
+        <v>605</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Hieu Salon Equipment Saigon</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>800</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Vietnam Customs tariff (20% import duty + 10% VAT) + sea LCL shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>180</v>
+      </c>
+      <c r="E4" t="n">
+        <v>107</v>
+      </c>
+      <c r="F4" t="n">
+        <v>287</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Excel Salon Furniture KL</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>500</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Malaysia customs clearing (5% duty + 10% SST) + Port Klang sea freight</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>350</v>
+      </c>
+      <c r="E5" t="n">
+        <v>212</v>
+      </c>
+      <c r="F5" t="n">
+        <v>562</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Excel Salon Furniture KL</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>950</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Port Klang sea LCL shipping + SST clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>180</v>
+      </c>
+      <c r="E6" t="n">
+        <v>106</v>
+      </c>
+      <c r="F6" t="n">
+        <v>286</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Premium Salon Supplies SG</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>800</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Singapore 9% GST + Keppel Port sea freight logistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>350</v>
+      </c>
+      <c r="E7" t="n">
+        <v>211</v>
+      </c>
+      <c r="F7" t="n">
+        <v>561</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Premium Salon Supplies SG</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Singapore sea LCL shipping + GST clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>180</v>
+      </c>
+      <c r="E8" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" t="n">
+        <v>250</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Takara Belmont HK Agent</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>700</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0% import duties/VAT, local truck logistics from Shenzhen port</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>350</v>
+      </c>
+      <c r="E9" t="n">
+        <v>150</v>
+      </c>
+      <c r="F9" t="n">
+        <v>500</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Takara Belmont HK Agent</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1300</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0% duties, sea LCL shipping + Kwai Chung port handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>180</v>
+      </c>
+      <c r="E10" t="n">
+        <v>75</v>
+      </c>
+      <c r="F10" t="n">
+        <v>255</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Macau Salon Distributor</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Macau 0% import duty, local logistics from HK port transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>350</v>
+      </c>
+      <c r="E11" t="n">
+        <v>150</v>
+      </c>
+      <c r="F11" t="n">
+        <v>500</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Macau Salon Distributor</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>1350</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Sea LCL shipping + Macau customs handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>180</v>
+      </c>
+      <c r="E12" t="n">
+        <v>113</v>
+      </c>
+      <c r="F12" t="n">
+        <v>293</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Taipei Salon Design Depot</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>600</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Taiwan Customs tariff (5% duty + 5% VAT) + Keelung port shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>350</v>
+      </c>
+      <c r="E13" t="n">
+        <v>215</v>
+      </c>
+      <c r="F13" t="n">
+        <v>565</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Taipei Salon Design Depot</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1100</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Taiwan sea LCL shipping + import customs clearance</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E14" t="n">
+        <v>128</v>
+      </c>
+      <c r="F14" t="n">
+        <v>308</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Takara Belmont Domestic</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>750</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Japan 10% consumption tax + Yokohama port shipping &amp; customs broker</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>350</v>
+      </c>
+      <c r="E15" t="n">
+        <v>235</v>
+      </c>
+      <c r="F15" t="n">
+        <v>585</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Takara Belmont Domestic</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Japan customs clearance + sea LCL logistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>180</v>
+      </c>
+      <c r="E16" t="n">
+        <v>142</v>
+      </c>
+      <c r="F16" t="n">
+        <v>322</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Takara Belmont Korea</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>750</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Korea Customs tariff (8% duty + 10% VAT) + Busan port LCL shipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>350</v>
+      </c>
+      <c r="E17" t="n">
+        <v>263</v>
+      </c>
+      <c r="F17" t="n">
+        <v>613</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Takara Belmont Korea</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Korea import clearance + sea freight logistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>180</v>
+      </c>
+      <c r="E18" t="n">
+        <v>188</v>
+      </c>
+      <c r="F18" t="n">
+        <v>368</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>EEM Salon Supplies Dubai</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>950</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>UAE Customs (5% duty + 5% VAT) + Jebel Ali port logistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>350</v>
+      </c>
+      <c r="E19" t="n">
+        <v>335</v>
+      </c>
+      <c r="F19" t="n">
+        <v>685</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>EEM Salon Supplies Dubai</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>1900</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Dubai LCL sea freight + local warehouse delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>180</v>
+      </c>
+      <c r="E20" t="n">
+        <v>257</v>
+      </c>
+      <c r="F20" t="n">
+        <v>437</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Comfortel Premium Australia</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>850</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Australian Border Force tariff (5% duty + 10% GST) + Port Botany freight</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>350</v>
+      </c>
+      <c r="E21" t="n">
+        <v>402</v>
+      </c>
+      <c r="F21" t="n">
+        <v>752</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Comfortel Premium Australia</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Australian Customs broker clearance + LCL sea cargo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Styling Chair</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Foshan Grand Hydraulic</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>180</v>
+      </c>
+      <c r="E22" t="n">
+        <v>133</v>
+      </c>
+      <c r="F22" t="n">
+        <v>313</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Bangkok Salon Supply</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>550</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Thailand Customs tariff (20% duty + 7% VAT) + Laem Chabang port logistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Shampoo Backwash Unit</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Premium Relax Basin Unit</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>350</v>
+      </c>
+      <c r="E23" t="n">
+        <v>254</v>
+      </c>
+      <c r="F23" t="n">
+        <v>604</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Bangkok Salon Supply</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>950</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Laem Chabang sea freight + customs clearance</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Brand / Item Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Wholesale Unit Price (USD)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Base Qty (4-Station Salon)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Total Cost (USD)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reference / Distributor Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Color &amp; Chemical</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Wella Koleston Perfect Permanent Color Tube (60ml)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Wella Professionals Distributor B2B Catalog 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Color &amp; Chemical</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wella Welloxon Perfect Developer (1000ml)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3" t="n">
+        <v>480</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Wella Professionals Distributor B2B Catalog 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Color &amp; Chemical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wella Blondor Multi-Blonde Bleach Powder (800g)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" t="n">
+        <v>500</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Wella Professionals Distributor B2B Catalog 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Color &amp; Chemical</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Olaplex Salon Intro Kit (Bond Multiplier No. 1 + Bond Perfector No. 2)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>150</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>750</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Olaplex Professional Partner B2B Pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Backwash Care</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kérastase Bain Chroma Respect (Color-treated, 1000ml)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>42</v>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>630</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>L'Oreal Division Professionnelle Trade Pricing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Backwash Care</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kérastase Bain Fluidealiste (Frizz control, 1000ml)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>42</v>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>630</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>L'Oreal Division Professionnelle Trade Pricing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Backwash Care</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kérastase Bain Densifique (Thinning/volume, 1000ml)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>42</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>420</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>L'Oreal Division Professionnelle Trade Pricing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Backwash Care</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kérastase Fondant Chroma Respect Conditioner (1000ml)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>48</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>576</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>L'Oreal Division Professionnelle Trade Pricing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Backwash Care</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kérastase Fondant Fluidealiste Conditioner (1000ml)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>48</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>576</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>L'Oreal Division Professionnelle Trade Pricing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Retail Stock</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Oribe Gold Lust Repair &amp; Restore Shampoo (250ml)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" t="n">
+        <v>980</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Oribe Salon Partner Program B2B Price List 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Retail Stock</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Oribe Gold Lust Repair &amp; Restore Conditioner (200ml)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>26</v>
+      </c>
+      <c r="D12" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Oribe Salon Partner Program B2B Price List 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Retail Stock</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Oribe Dry Texturizing Spray (300ml)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" t="n">
+        <v>30</v>
+      </c>
+      <c r="E13" t="n">
+        <v>720</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Oribe Salon Partner Program B2B Price List 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Retail Stock</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kérastase Elixir Ultime Hair Oil (100ml)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>L'Oreal Division Professionnelle Trade Pricing 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Backstation Essentials</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Oribe Royal Blowout Heat Styling Spray (175ml)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>34</v>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" t="n">
+        <v>510</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Oribe Salon Partner Program B2B Price List 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Backstation Essentials</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Oribe Gold Lust Dry Shampoo (250ml)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>24</v>
+      </c>
+      <c r="D16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" t="n">
+        <v>480</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Oribe Salon Partner Program B2B Price List 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Backstation Essentials</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Miscellaneous color bowls, brushes, foils, gloves, capes, towels (Lot)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Salon Essentials Wholesale Distributor Lot Price 2025</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>